<commit_message>
B1: 2026-04-01 — 107 plays
</commit_message>
<xml_diff>
--- a/daily/2026-04-01.xlsx
+++ b/daily/2026-04-01.xlsx
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>19.5</v>
+        <v>18.5</v>
       </c>
       <c r="E5" t="n">
         <v>21.3</v>
@@ -854,10 +854,10 @@
         <v>80</v>
       </c>
       <c r="P5" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.6</v>
+        <v>1.6</v>
       </c>
       <c r="R5" t="n">
         <v>2.1</v>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="E9" t="n">
         <v>13.3</v>
@@ -1179,13 +1179,13 @@
         <v>7.2</v>
       </c>
       <c r="O9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="P9" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.4</v>
+        <v>-0.6</v>
       </c>
       <c r="R9" t="n">
         <v>4.1</v>
@@ -1538,7 +1538,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jevon Carter</t>
+          <t>Franz Wagner</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1548,73 +1548,73 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Guard</t>
+          <t>Forward</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>8.5</v>
+        <v>11.5</v>
       </c>
       <c r="E14" t="n">
-        <v>4.7</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>6.2</v>
+        <v>11.6</v>
       </c>
       <c r="G14" t="n">
-        <v>8.6</v>
+        <v>18.2</v>
       </c>
       <c r="H14" t="n">
-        <v>7.3</v>
+        <v>21</v>
       </c>
       <c r="I14" t="n">
-        <v>6.7</v>
+        <v>21.4</v>
       </c>
       <c r="J14" t="n">
-        <v>20.6</v>
+        <v>26.3</v>
       </c>
       <c r="K14" t="n">
-        <v>17.7</v>
+        <v>31.9</v>
       </c>
       <c r="L14" t="n">
-        <v>41.6</v>
+        <v>49.7</v>
       </c>
       <c r="M14" t="n">
-        <v>35.1</v>
+        <v>48.1</v>
       </c>
       <c r="N14" t="n">
-        <v>4.9</v>
+        <v>8.4</v>
       </c>
       <c r="O14" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="P14" t="n">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="Q14" t="n">
-        <v>-1.8</v>
+        <v>9.9</v>
       </c>
       <c r="R14" t="n">
-        <v>-0.5</v>
+        <v>-9.800000000000001</v>
       </c>
       <c r="S14" t="n">
-        <v>6.5</v>
+        <v>1.6</v>
       </c>
       <c r="T14" t="n">
-        <v>2.9</v>
+        <v>-5.6</v>
       </c>
       <c r="U14" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="V14" t="n">
         <v>6</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>9.8 (4g)</t>
+          <t>25.8 (5g)</t>
         </is>
       </c>
       <c r="X14" t="n">
-        <v>17.9</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="15">
@@ -2438,7 +2438,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="E25" t="n">
         <v>12.3</v>
@@ -2474,10 +2474,10 @@
         <v>40</v>
       </c>
       <c r="P25" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="Q25" t="n">
-        <v>-0.9</v>
+        <v>-1.9</v>
       </c>
       <c r="R25" t="n">
         <v>2.2</v>
@@ -3966,7 +3966,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kevin Durant</t>
+          <t>Jabari Smith Jr.</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3980,55 +3980,55 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>25.5</v>
+        <v>14.5</v>
       </c>
       <c r="E44" t="n">
-        <v>24</v>
+        <v>18.7</v>
       </c>
       <c r="F44" t="n">
-        <v>28.4</v>
+        <v>15.6</v>
       </c>
       <c r="G44" t="n">
-        <v>26.2</v>
+        <v>17</v>
       </c>
       <c r="H44" t="n">
-        <v>25.4</v>
+        <v>16.6</v>
       </c>
       <c r="I44" t="n">
-        <v>25.2</v>
+        <v>15.9</v>
       </c>
       <c r="J44" t="n">
-        <v>36.3</v>
+        <v>38.2</v>
       </c>
       <c r="K44" t="n">
         <v>35.7</v>
       </c>
       <c r="L44" t="n">
-        <v>54.3</v>
+        <v>42.5</v>
       </c>
       <c r="M44" t="n">
-        <v>53</v>
+        <v>48.3</v>
       </c>
       <c r="N44" t="n">
-        <v>6.8</v>
+        <v>5.1</v>
       </c>
       <c r="O44" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="P44" t="n">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="Q44" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="R44" t="n">
         <v>-0.3</v>
       </c>
-      <c r="R44" t="n">
-        <v>3.2</v>
-      </c>
       <c r="S44" t="n">
-        <v>1.3</v>
+        <v>-5.8</v>
       </c>
       <c r="T44" t="n">
-        <v>0.6</v>
+        <v>2.5</v>
       </c>
       <c r="U44" t="n">
         <v>23</v>
@@ -4036,15 +4036,19 @@
       <c r="V44" t="n">
         <v>14</v>
       </c>
-      <c r="W44" t="inlineStr"/>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>11.0 (3g)</t>
+        </is>
+      </c>
       <c r="X44" t="n">
-        <v>13.1</v>
+        <v>-7.6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jabari Smith Jr.</t>
+          <t>Kevin Durant</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4058,55 +4062,55 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>16.5</v>
+        <v>25.5</v>
       </c>
       <c r="E45" t="n">
-        <v>18.7</v>
+        <v>24</v>
       </c>
       <c r="F45" t="n">
-        <v>15.6</v>
+        <v>28.4</v>
       </c>
       <c r="G45" t="n">
-        <v>17</v>
+        <v>26.2</v>
       </c>
       <c r="H45" t="n">
-        <v>16.6</v>
+        <v>25.4</v>
       </c>
       <c r="I45" t="n">
-        <v>15.9</v>
+        <v>25.2</v>
       </c>
       <c r="J45" t="n">
-        <v>38.2</v>
+        <v>36.3</v>
       </c>
       <c r="K45" t="n">
         <v>35.7</v>
       </c>
       <c r="L45" t="n">
-        <v>42.5</v>
+        <v>54.3</v>
       </c>
       <c r="M45" t="n">
-        <v>48.3</v>
+        <v>53</v>
       </c>
       <c r="N45" t="n">
-        <v>5.1</v>
+        <v>6.8</v>
       </c>
       <c r="O45" t="n">
         <v>50</v>
       </c>
       <c r="P45" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q45" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="R45" t="n">
-        <v>-0.3</v>
+        <v>3.2</v>
       </c>
       <c r="S45" t="n">
-        <v>-5.8</v>
+        <v>1.3</v>
       </c>
       <c r="T45" t="n">
-        <v>2.5</v>
+        <v>0.6</v>
       </c>
       <c r="U45" t="n">
         <v>23</v>
@@ -4114,13 +4118,9 @@
       <c r="V45" t="n">
         <v>14</v>
       </c>
-      <c r="W45" t="inlineStr">
-        <is>
-          <t>11.0 (3g)</t>
-        </is>
-      </c>
+      <c r="W45" t="inlineStr"/>
       <c r="X45" t="n">
-        <v>-7.6</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="46">
@@ -4208,7 +4208,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tari Eason</t>
+          <t>Gary Trent Jr.</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4218,79 +4218,79 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Forward</t>
+          <t>Guard</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>9.5</v>
+        <v>15.5</v>
       </c>
       <c r="E47" t="n">
-        <v>16</v>
+        <v>22.3</v>
       </c>
       <c r="F47" t="n">
-        <v>11</v>
+        <v>17.4</v>
       </c>
       <c r="G47" t="n">
-        <v>9.1</v>
+        <v>11.9</v>
       </c>
       <c r="H47" t="n">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I47" t="n">
-        <v>9.6</v>
+        <v>7.5</v>
       </c>
       <c r="J47" t="n">
-        <v>24.6</v>
+        <v>22.1</v>
       </c>
       <c r="K47" t="n">
-        <v>27.8</v>
+        <v>16.5</v>
       </c>
       <c r="L47" t="n">
-        <v>31.6</v>
+        <v>37.9</v>
       </c>
       <c r="M47" t="n">
-        <v>36.9</v>
+        <v>32.7</v>
       </c>
       <c r="N47" t="n">
-        <v>5.3</v>
+        <v>10.7</v>
       </c>
       <c r="O47" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="P47" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.1</v>
+        <v>-8</v>
       </c>
       <c r="R47" t="n">
-        <v>1.4</v>
+        <v>9.9</v>
       </c>
       <c r="S47" t="n">
-        <v>-5.3</v>
+        <v>5.2</v>
       </c>
       <c r="T47" t="n">
-        <v>-3.3</v>
+        <v>5.6</v>
       </c>
       <c r="U47" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="V47" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>9.0 (3g)</t>
+          <t>8.7 (3g)</t>
         </is>
       </c>
       <c r="X47" t="n">
-        <v>-3.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Gary Trent Jr.</t>
+          <t>Tari Eason</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -4300,73 +4300,73 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Guard</t>
+          <t>Forward</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>13.5</v>
+        <v>9.5</v>
       </c>
       <c r="E48" t="n">
-        <v>22.3</v>
+        <v>16</v>
       </c>
       <c r="F48" t="n">
-        <v>17.4</v>
+        <v>11</v>
       </c>
       <c r="G48" t="n">
-        <v>11.9</v>
+        <v>9.1</v>
       </c>
       <c r="H48" t="n">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I48" t="n">
-        <v>7.5</v>
+        <v>9.6</v>
       </c>
       <c r="J48" t="n">
-        <v>22.1</v>
+        <v>24.6</v>
       </c>
       <c r="K48" t="n">
-        <v>16.5</v>
+        <v>27.8</v>
       </c>
       <c r="L48" t="n">
-        <v>37.9</v>
+        <v>31.6</v>
       </c>
       <c r="M48" t="n">
-        <v>32.7</v>
+        <v>36.9</v>
       </c>
       <c r="N48" t="n">
-        <v>10.7</v>
+        <v>5.3</v>
       </c>
       <c r="O48" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="P48" t="n">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="Q48" t="n">
-        <v>-6</v>
+        <v>0.1</v>
       </c>
       <c r="R48" t="n">
-        <v>9.9</v>
+        <v>1.4</v>
       </c>
       <c r="S48" t="n">
-        <v>5.2</v>
+        <v>-5.3</v>
       </c>
       <c r="T48" t="n">
-        <v>5.6</v>
+        <v>-3.3</v>
       </c>
       <c r="U48" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="V48" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>8.7 (3g)</t>
+          <t>9.0 (3g)</t>
         </is>
       </c>
       <c r="X48" t="n">
-        <v>7.9</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="49">
@@ -5418,7 +5418,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DeMar DeRozan</t>
+          <t>RJ Barrett</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5428,79 +5428,75 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Guard</t>
+          <t>Forward</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>18.5</v>
+        <v>22.5</v>
       </c>
       <c r="E62" t="n">
-        <v>20.7</v>
+        <v>22</v>
       </c>
       <c r="F62" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G62" t="n">
-        <v>20.6</v>
+        <v>20.8</v>
       </c>
       <c r="H62" t="n">
-        <v>17.4</v>
+        <v>19.9</v>
       </c>
       <c r="I62" t="n">
-        <v>17.6</v>
+        <v>19</v>
       </c>
       <c r="J62" t="n">
-        <v>30.9</v>
+        <v>30.3</v>
       </c>
       <c r="K62" t="n">
-        <v>28.7</v>
+        <v>29.8</v>
       </c>
       <c r="L62" t="n">
-        <v>49.7</v>
+        <v>54.5</v>
       </c>
       <c r="M62" t="n">
-        <v>45.8</v>
+        <v>49</v>
       </c>
       <c r="N62" t="n">
-        <v>13.8</v>
+        <v>5.3</v>
       </c>
       <c r="O62" t="n">
         <v>50</v>
       </c>
       <c r="P62" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="Q62" t="n">
-        <v>-0.9</v>
+        <v>-3.5</v>
       </c>
       <c r="R62" t="n">
-        <v>-0.6</v>
+        <v>2</v>
       </c>
       <c r="S62" t="n">
-        <v>3.9</v>
+        <v>5.5</v>
       </c>
       <c r="T62" t="n">
-        <v>2.2</v>
+        <v>0.5</v>
       </c>
       <c r="U62" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="V62" t="n">
-        <v>25</v>
-      </c>
-      <c r="W62" t="inlineStr">
-        <is>
-          <t>23.0 (3g)</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="W62" t="inlineStr"/>
       <c r="X62" t="n">
-        <v>-2.2</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Collin Murray-Boyles</t>
+          <t>DeMar DeRozan</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5510,75 +5506,79 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Forward</t>
+          <t>Guard</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>11.5</v>
+        <v>18.5</v>
       </c>
       <c r="E63" t="n">
-        <v>11</v>
+        <v>20.7</v>
       </c>
       <c r="F63" t="n">
-        <v>9.199999999999999</v>
+        <v>17</v>
       </c>
       <c r="G63" t="n">
-        <v>8.800000000000001</v>
+        <v>20.6</v>
       </c>
       <c r="H63" t="n">
-        <v>9.4</v>
+        <v>17.4</v>
       </c>
       <c r="I63" t="n">
-        <v>8.699999999999999</v>
+        <v>17.6</v>
       </c>
       <c r="J63" t="n">
-        <v>21.6</v>
+        <v>30.9</v>
       </c>
       <c r="K63" t="n">
-        <v>25.1</v>
+        <v>28.7</v>
       </c>
       <c r="L63" t="n">
-        <v>71.40000000000001</v>
+        <v>49.7</v>
       </c>
       <c r="M63" t="n">
-        <v>59.8</v>
+        <v>45.8</v>
       </c>
       <c r="N63" t="n">
-        <v>4.6</v>
+        <v>13.8</v>
       </c>
       <c r="O63" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="P63" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="Q63" t="n">
-        <v>-2.8</v>
+        <v>-0.9</v>
       </c>
       <c r="R63" t="n">
-        <v>0.5</v>
+        <v>-0.6</v>
       </c>
       <c r="S63" t="n">
-        <v>11.6</v>
+        <v>3.9</v>
       </c>
       <c r="T63" t="n">
-        <v>-3.5</v>
+        <v>2.2</v>
       </c>
       <c r="U63" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="V63" t="n">
-        <v>15</v>
-      </c>
-      <c r="W63" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>23.0 (3g)</t>
+        </is>
+      </c>
       <c r="X63" t="n">
-        <v>0</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ja'Kobe Walter</t>
+          <t>Collin Murray-Boyles</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5588,20 +5588,20 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Guard</t>
+          <t>Forward</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="E64" t="n">
-        <v>10.7</v>
+        <v>11</v>
       </c>
       <c r="F64" t="n">
-        <v>11.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G64" t="n">
-        <v>11.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H64" t="n">
         <v>9.4</v>
@@ -5610,53 +5610,53 @@
         <v>8.699999999999999</v>
       </c>
       <c r="J64" t="n">
-        <v>23.9</v>
+        <v>21.6</v>
       </c>
       <c r="K64" t="n">
-        <v>21.9</v>
+        <v>25.1</v>
       </c>
       <c r="L64" t="n">
-        <v>55.1</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="M64" t="n">
-        <v>41.4</v>
+        <v>59.8</v>
       </c>
       <c r="N64" t="n">
-        <v>6.4</v>
+        <v>4.6</v>
       </c>
       <c r="O64" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="P64" t="n">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="Q64" t="n">
-        <v>-1.8</v>
+        <v>-2.8</v>
       </c>
       <c r="R64" t="n">
-        <v>2.9</v>
+        <v>0.5</v>
       </c>
       <c r="S64" t="n">
-        <v>13.7</v>
+        <v>11.6</v>
       </c>
       <c r="T64" t="n">
-        <v>2</v>
+        <v>-3.5</v>
       </c>
       <c r="U64" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="V64" t="n">
         <v>15</v>
       </c>
       <c r="W64" t="inlineStr"/>
       <c r="X64" t="n">
-        <v>-32.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RJ Barrett</t>
+          <t>Ja'Kobe Walter</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -5666,69 +5666,69 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Forward</t>
+          <t>Guard</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>21.5</v>
+        <v>10.5</v>
       </c>
       <c r="E65" t="n">
-        <v>22</v>
+        <v>10.7</v>
       </c>
       <c r="F65" t="n">
-        <v>21</v>
+        <v>11.6</v>
       </c>
       <c r="G65" t="n">
-        <v>20.8</v>
+        <v>11.8</v>
       </c>
       <c r="H65" t="n">
-        <v>19.9</v>
+        <v>9.4</v>
       </c>
       <c r="I65" t="n">
-        <v>19</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J65" t="n">
-        <v>30.3</v>
+        <v>23.9</v>
       </c>
       <c r="K65" t="n">
-        <v>29.8</v>
+        <v>21.9</v>
       </c>
       <c r="L65" t="n">
-        <v>54.5</v>
+        <v>55.1</v>
       </c>
       <c r="M65" t="n">
-        <v>49</v>
+        <v>41.4</v>
       </c>
       <c r="N65" t="n">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
       <c r="O65" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="P65" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="Q65" t="n">
-        <v>-2.5</v>
+        <v>-1.8</v>
       </c>
       <c r="R65" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="S65" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="T65" t="n">
         <v>2</v>
       </c>
-      <c r="S65" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="T65" t="n">
-        <v>0.5</v>
-      </c>
       <c r="U65" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="V65" t="n">
         <v>15</v>
       </c>
       <c r="W65" t="inlineStr"/>
       <c r="X65" t="n">
-        <v>-5</v>
+        <v>-32.6</v>
       </c>
     </row>
     <row r="66">
@@ -6384,7 +6384,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="E74" t="n">
         <v>14</v>
@@ -6417,13 +6417,13 @@
         <v>7.1</v>
       </c>
       <c r="O74" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="P74" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="Q74" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="R74" t="n">
         <v>-0.1</v>
@@ -6946,7 +6946,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18.5</v>
+        <v>19.5</v>
       </c>
       <c r="E81" t="n">
         <v>22.7</v>
@@ -6982,10 +6982,10 @@
         <v>70</v>
       </c>
       <c r="P81" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="Q81" t="n">
-        <v>-3.4</v>
+        <v>-4.4</v>
       </c>
       <c r="R81" t="n">
         <v>6.7</v>
@@ -9373,10 +9373,10 @@
         <v>3.7</v>
       </c>
       <c r="J3" t="n">
-        <v>3.15</v>
+        <v>2.9</v>
       </c>
       <c r="K3" t="n">
-        <v>1.333</v>
+        <v>1.385</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
@@ -9421,10 +9421,10 @@
         <v>1.1</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="K4" t="n">
-        <v>1.364</v>
+        <v>1.345</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
@@ -9454,10 +9454,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.635</v>
+        <v>0.667</v>
       </c>
       <c r="F5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -9466,17 +9466,17 @@
         <v>24</v>
       </c>
       <c r="I5" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="J5" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="K5" t="n">
-        <v>1.408</v>
+        <v>1.385</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Recent scoring trending up 2.1 pts (L5 vs L30) — supports the OVER. TS% shifts +6.1% in this matchup; FG% +6.4% trending (L10 vs L30). Opponent is below-average defense (#18) at slow pace (#29). 7/10 signals agree — Volume, HR L30, HR L10, Trend support the OVER; H2H, Pace, Min Trend dissent. Projection model targets 24.0 pts (4.5 pts above line; 63% blended confidence [T2]). Risk: high variance (σ=7.1) makes the outcome difficult to call with confidence.</t>
+          <t>Recent scoring trending up 2.1 pts (L5 vs L30) — supports the OVER. TS% shifts +6.1% in this matchup; FG% +6.4% trending (L10 vs L30). Opponent is below-average defense (#18) at slow pace (#29). 8/10 signals agree — Volume, HR L30, HR L10, Trend support the OVER; Pace, Min Trend dissent. Projection model targets 24.0 pts (5.5 pts above line; 66% blended confidence [T2]). Risk: high variance (σ=7.1) makes the outcome difficult to call with confidence.</t>
         </is>
       </c>
     </row>
@@ -9517,10 +9517,10 @@
         <v>5.1</v>
       </c>
       <c r="J6" t="n">
-        <v>3.05</v>
+        <v>2.75</v>
       </c>
       <c r="K6" t="n">
-        <v>1.357</v>
+        <v>1.417</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
@@ -9565,10 +9565,10 @@
         <v>5.9</v>
       </c>
       <c r="J7" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
       <c r="K7" t="n">
-        <v>1.345</v>
+        <v>1.435</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
@@ -9646,29 +9646,29 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.54</v>
+        <v>0.552</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="I9" t="n">
-        <v>0.5</v>
+        <v>1.6</v>
       </c>
       <c r="J9" t="n">
-        <v>2.85</v>
+        <v>2.7</v>
       </c>
       <c r="K9" t="n">
-        <v>1.4</v>
+        <v>1.435</v>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Recent scoring trending up 4.1 pts (L5 vs L30) — marginally supports the UNDER. FG% +3.8% trending (L10 vs L30). Opponent is below-average defense (#18) at slow pace (#29). Mixed signals: 2/10 agree (Context, Pace); counter-signals: Volume, HR L30, HR L10. Projection model targets 11.0 pts (0.5 pts below line; 53% blended confidence [T3]). Risk: high variance (σ=7.2) makes the outcome difficult to call with confidence.</t>
+          <t>Recent scoring trending up 4.1 pts (L5 vs L30) — marginally supports the UNDER. FG% +3.8% trending (L10 vs L30). Opponent is below-average defense (#18) at slow pace (#29). Mixed signals: 5/10 agree (Volume, HR L30, Context); counter-signals: HR L10, Trend, Defense. Projection model targets 10.9 pts (1.6 pts below line; 55% blended confidence [T3]). Risk: high variance (σ=7.2) makes the outcome difficult to call with confidence.</t>
         </is>
       </c>
     </row>
@@ -9709,10 +9709,10 @@
         <v>0.7</v>
       </c>
       <c r="J10" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="K10" t="n">
-        <v>1.408</v>
+        <v>1.385</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
@@ -9805,10 +9805,10 @@
         <v>5.1</v>
       </c>
       <c r="J12" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="K12" t="n">
-        <v>1.408</v>
+        <v>1.385</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
@@ -9867,7 +9867,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jevon Carter</t>
+          <t>Franz Wagner</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9886,29 +9886,29 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.556</v>
+        <v>0.726</v>
       </c>
       <c r="F14" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>10.7</v>
+        <v>18.8</v>
       </c>
       <c r="I14" t="n">
-        <v>2.2</v>
+        <v>7.3</v>
       </c>
       <c r="J14" t="n">
-        <v>2.1</v>
+        <v>1.87</v>
       </c>
       <c r="K14" t="n">
-        <v>1.69</v>
+        <v>1.893</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Low scoring variance (σ=4.9) — highly predictable output near line — marginally supports the OVER. H2H avg 3.1 pts above season L30; TS% shifts +17.9% in this matchup. Opponent is below-average defense (#20) at above-average pace (#6). Mixed signals: 5/10 agree (Defense, H2H, Pace); counter-signals: Volume, HR L30, HR L10. Projection model targets 10.7 pts (2.2 pts above line; 55% blended confidence [T3]). Risk: only 37% hit rate over L30 suggests the line may be set fairly.</t>
+          <t>Wagner averages 25.8 pts in 5 meetings (+14.3 vs line) — supports the OVER. H2H avg 4.4 pts above season L30; Minutes down 5.6 recently (L10=26.3 vs L30=31.9). Opponent is weak defense (#24) at above-average pace (#6). 8/10 signals agree — Volume, HR L30, HR L10, Context support the OVER; Trend, Min Trend dissent. Projection model targets 18.8 pts (7.3 pts above line; 72% blended confidence [T3]). Risk: L3 has dropped to 11.0 (10.4 below L30) — deepening slump makes the over vulnerable.</t>
         </is>
       </c>
     </row>
@@ -9949,10 +9949,10 @@
         <v>3.5</v>
       </c>
       <c r="J15" t="n">
-        <v>1.943</v>
+        <v>1.901</v>
       </c>
       <c r="K15" t="n">
-        <v>1.82</v>
+        <v>1.862</v>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
@@ -10045,10 +10045,10 @@
         <v>1.9</v>
       </c>
       <c r="J17" t="n">
-        <v>1.877</v>
+        <v>1.87</v>
       </c>
       <c r="K17" t="n">
-        <v>1.877</v>
+        <v>1.893</v>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
@@ -10093,10 +10093,10 @@
         <v>1.1</v>
       </c>
       <c r="J18" t="n">
-        <v>1.909</v>
+        <v>1.926</v>
       </c>
       <c r="K18" t="n">
-        <v>1.847</v>
+        <v>1.833</v>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
@@ -10141,10 +10141,10 @@
         <v>1.7</v>
       </c>
       <c r="J19" t="n">
-        <v>1.971</v>
+        <v>1.917</v>
       </c>
       <c r="K19" t="n">
-        <v>1.8</v>
+        <v>1.84</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
@@ -10189,10 +10189,10 @@
         <v>3.3</v>
       </c>
       <c r="J20" t="n">
-        <v>1.87</v>
+        <v>1.952</v>
       </c>
       <c r="K20" t="n">
-        <v>1.893</v>
+        <v>1.813</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
@@ -10285,10 +10285,10 @@
         <v>3.4</v>
       </c>
       <c r="J22" t="n">
-        <v>1.952</v>
+        <v>1.98</v>
       </c>
       <c r="K22" t="n">
-        <v>1.813</v>
+        <v>1.787</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
@@ -10333,10 +10333,10 @@
         <v>4.2</v>
       </c>
       <c r="J23" t="n">
-        <v>1.84</v>
+        <v>1.971</v>
       </c>
       <c r="K23" t="n">
-        <v>1.917</v>
+        <v>1.8</v>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
@@ -10381,10 +10381,10 @@
         <v>0.8</v>
       </c>
       <c r="J24" t="n">
+        <v>1.893</v>
+      </c>
+      <c r="K24" t="n">
         <v>1.87</v>
-      </c>
-      <c r="K24" t="n">
-        <v>1.893</v>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
@@ -10414,10 +10414,10 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.537</v>
+        <v>0.514</v>
       </c>
       <c r="F25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -10426,17 +10426,17 @@
         <v>12.9</v>
       </c>
       <c r="I25" t="n">
-        <v>1.4</v>
+        <v>0.4</v>
       </c>
       <c r="J25" t="n">
-        <v>1.917</v>
+        <v>1.952</v>
       </c>
       <c r="K25" t="n">
-        <v>1.84</v>
+        <v>1.813</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Vukcevic averages 14.8 pts in 4 meetings (+3.3 vs line) — supports the OVER. H2H avg 4.2 pts above season L30; TS% shifts +4.1% in this matchup. Opponent is below-average defense (#21) at slow pace (#23). 6/10 signals agree — Trend, Context, Defense, H2H support the OVER; Volume, HR L30, HR L10 dissent. Projection model targets 12.9 pts (1.4 pts above line; 53% blended confidence [T3]).</t>
+          <t>Vukcevic averages 14.8 pts in 4 meetings (+2.3 vs line) — marginally supports the OVER. H2H avg 4.2 pts above season L30; TS% shifts +4.1% in this matchup. Opponent is below-average defense (#21) at slow pace (#23). Mixed signals: 5/10 agree (Trend, Defense, H2H); counter-signals: Volume, HR L30, HR L10. Projection model targets 12.9 pts (0.4 pts above line; 51% blended confidence [T3]).</t>
         </is>
       </c>
     </row>
@@ -10477,10 +10477,10 @@
         <v>1.3</v>
       </c>
       <c r="J26" t="n">
-        <v>1.943</v>
+        <v>1.926</v>
       </c>
       <c r="K26" t="n">
-        <v>1.82</v>
+        <v>1.833</v>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
@@ -10621,10 +10621,10 @@
         <v>2.9</v>
       </c>
       <c r="J29" t="n">
-        <v>1.769</v>
+        <v>1.699</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
@@ -10669,10 +10669,10 @@
         <v>5.2</v>
       </c>
       <c r="J30" t="n">
-        <v>1.952</v>
+        <v>1.943</v>
       </c>
       <c r="K30" t="n">
-        <v>1.813</v>
+        <v>1.82</v>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
@@ -10717,10 +10717,10 @@
         <v>1.8</v>
       </c>
       <c r="J31" t="n">
-        <v>1.813</v>
+        <v>1.87</v>
       </c>
       <c r="K31" t="n">
-        <v>1.952</v>
+        <v>1.893</v>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
@@ -10909,10 +10909,10 @@
         <v>0.7</v>
       </c>
       <c r="J35" t="n">
-        <v>1.787</v>
+        <v>1.813</v>
       </c>
       <c r="K35" t="n">
-        <v>1.98</v>
+        <v>1.962</v>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
@@ -11005,10 +11005,10 @@
         <v>0.3</v>
       </c>
       <c r="J37" t="n">
-        <v>1.82</v>
+        <v>1.813</v>
       </c>
       <c r="K37" t="n">
-        <v>1.943</v>
+        <v>1.952</v>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
@@ -11053,10 +11053,10 @@
         <v>2</v>
       </c>
       <c r="J38" t="n">
-        <v>1.952</v>
+        <v>1.943</v>
       </c>
       <c r="K38" t="n">
-        <v>1.813</v>
+        <v>1.82</v>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
@@ -11101,10 +11101,10 @@
         <v>4.6</v>
       </c>
       <c r="J39" t="n">
-        <v>1.87</v>
+        <v>1.901</v>
       </c>
       <c r="K39" t="n">
-        <v>1.87</v>
+        <v>1.847</v>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
@@ -11149,10 +11149,10 @@
         <v>12.1</v>
       </c>
       <c r="J40" t="n">
-        <v>3.1</v>
+        <v>2.85</v>
       </c>
       <c r="K40" t="n">
-        <v>1.345</v>
+        <v>1.4</v>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
@@ -11197,10 +11197,10 @@
         <v>2.3</v>
       </c>
       <c r="J41" t="n">
-        <v>1.87</v>
+        <v>1.901</v>
       </c>
       <c r="K41" t="n">
-        <v>1.87</v>
+        <v>1.833</v>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
@@ -11245,10 +11245,10 @@
         <v>3.1</v>
       </c>
       <c r="J42" t="n">
-        <v>1.8</v>
+        <v>2.55</v>
       </c>
       <c r="K42" t="n">
-        <v>1.943</v>
+        <v>1.476</v>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
@@ -11293,10 +11293,10 @@
         <v>3.1</v>
       </c>
       <c r="J43" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="K43" t="n">
-        <v>1.435</v>
+        <v>1.385</v>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
@@ -11307,7 +11307,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kevin Durant</t>
+          <t>Jabari Smith Jr.</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -11317,45 +11317,45 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.571</v>
+        <v>0.593</v>
       </c>
       <c r="F44" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>27.9</v>
+        <v>11.5</v>
       </c>
       <c r="I44" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>1.87</v>
+        <v>1.769</v>
       </c>
       <c r="K44" t="n">
-        <v>1.87</v>
+        <v>1.952</v>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Recent scoring trending up 3.2 pts (L5 vs L30) — supports the OVER. Opponent is weak defense (#23) at moderate pace (#14). 6/10 signals agree — Trend, Context, Defense, Pace support the OVER; Volume, HR L30, HR L10 dissent. Projection model targets 27.9 pts (2.4 pts above line; 57% blended confidence [T2]).</t>
+          <t>Jr. averages 11.0 pts in 3 meetings (-3.5 vs line) — marginally supports the UNDER. H2H avg 4.9 pts below season L30; TS% shifts -7.6% in this matchup. Opponent is weak defense (#23) at moderate pace (#14). Mixed signals: 3/10 agree (Trend, H2H, FG Trend); counter-signals: Volume, HR L30, HR L10. Projection model targets 11.5 pts (3.0 pts below line; 59% blended confidence [T3]). Risk: 60% over-rate on L30 suggests scoring tendency that could threaten the under.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jabari Smith Jr.</t>
+          <t>Kevin Durant</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -11365,7 +11365,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -11374,7 +11374,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.629</v>
+        <v>0.571</v>
       </c>
       <c r="F45" t="n">
         <v>6</v>
@@ -11383,10 +11383,10 @@
         <v>1</v>
       </c>
       <c r="H45" t="n">
-        <v>11.6</v>
+        <v>27.9</v>
       </c>
       <c r="I45" t="n">
-        <v>4.9</v>
+        <v>2.4</v>
       </c>
       <c r="J45" t="n">
         <v>1.769</v>
@@ -11396,7 +11396,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Jr. averages 11.0 pts in 3 meetings (-5.5 vs line) — supports the UNDER. H2H avg 4.9 pts below season L30; TS% shifts -7.6% in this matchup. Opponent is weak defense (#23) at moderate pace (#14). 6/10 signals agree — Volume, HR L30, Trend, Context support the UNDER; HR L10, Defense, Pace dissent. Projection model targets 11.6 pts (4.9 pts below line; 62% blended confidence [T2]).</t>
+          <t>Recent scoring trending up 3.2 pts (L5 vs L30) — supports the OVER. Opponent is weak defense (#23) at moderate pace (#14). 6/10 signals agree — Trend, Context, Defense, Pace support the OVER; Volume, HR L30, HR L10 dissent. Projection model targets 27.9 pts (2.4 pts above line; 57% blended confidence [T2]).</t>
         </is>
       </c>
     </row>
@@ -11437,10 +11437,10 @@
         <v>3.1</v>
       </c>
       <c r="J46" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K46" t="n">
         <v>1.952</v>
-      </c>
-      <c r="K46" t="n">
-        <v>1.8</v>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
@@ -11451,7 +11451,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tari Eason</t>
+          <t>Gary Trent Jr.</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -11470,36 +11470,36 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.546</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="F47" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>7.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I47" t="n">
-        <v>1.9</v>
+        <v>6.8</v>
       </c>
       <c r="J47" t="n">
-        <v>1.909</v>
+        <v>2.7</v>
       </c>
       <c r="K47" t="n">
-        <v>1.833</v>
+        <v>1.435</v>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Eason's L30 average of 9.6 pts vs the 9.5 line — marginally supports the UNDER. TS% shifts -3.7% in this matchup; FG% -5.3% trending (L10 vs L30). Opponent is weak defense (#23) at moderate pace (#14). Mixed signals: 5/10 agree (HR L30, Context, H2H); counter-signals: Volume, HR L10, Trend. Projection model targets 7.6 pts (1.9 pts below line; 54% blended confidence [T3]). Risk: L3 has surged to 16.0 after a 11-pt outing (6.4 above L30) — momentum could push over the under line.</t>
+          <t>Jr.'s L30 of 7.5 pts sits 8.0 below the 15.5 line — supports the UNDER. TS% shifts +7.9% in this matchup; FG% +5.2% trending (L10 vs L30). Opponent is elite defense (#5) at slow pace (#22). 7/10 signals agree — Volume, HR L30, HR L10, Context support the UNDER; Trend, FG Trend, Min Trend dissent. Projection model targets 8.7 pts (6.8 pts below line; 69% blended confidence [T3]). Risk: L3 has surged to 22.3 after a 15-pt outing (14.8 above L30) — momentum could push over the under line.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Gary Trent Jr.</t>
+          <t>Tari Eason</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -11518,29 +11518,29 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.642</v>
+        <v>0.546</v>
       </c>
       <c r="F48" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>8.699999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="I48" t="n">
-        <v>4.8</v>
+        <v>1.9</v>
       </c>
       <c r="J48" t="n">
-        <v>3</v>
+        <v>1.952</v>
       </c>
       <c r="K48" t="n">
-        <v>1.364</v>
+        <v>1.8</v>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Recent scoring trending up 9.9 pts (L5 vs L30) — supports the UNDER. TS% shifts +7.9% in this matchup; FG% +5.2% trending (L10 vs L30). Opponent is elite defense (#5) at slow pace (#22). 7/10 signals agree — Volume, HR L30, HR L10, Context support the UNDER; Trend, FG Trend, Min Trend dissent. Projection model targets 8.7 pts (4.8 pts below line; 64% blended confidence [T3]). Risk: L3 has surged to 22.3 after a 15-pt outing (14.8 above L30) — momentum could push over the under line.</t>
+          <t>Eason's L30 average of 9.6 pts vs the 9.5 line — marginally supports the UNDER. TS% shifts -3.7% in this matchup; FG% -5.3% trending (L10 vs L30). Opponent is weak defense (#23) at moderate pace (#14). Mixed signals: 5/10 agree (HR L30, Context, H2H); counter-signals: Volume, HR L10, Trend. Projection model targets 7.6 pts (1.9 pts below line; 54% blended confidence [T3]). Risk: L3 has surged to 16.0 after a 11-pt outing (6.4 above L30) — momentum could push over the under line.</t>
         </is>
       </c>
     </row>
@@ -11581,10 +11581,10 @@
         <v>1.1</v>
       </c>
       <c r="J49" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="K49" t="n">
-        <v>1.73</v>
+        <v>1.719</v>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
@@ -11725,10 +11725,10 @@
         <v>1.5</v>
       </c>
       <c r="J52" t="n">
-        <v>3.15</v>
+        <v>3.05</v>
       </c>
       <c r="K52" t="n">
-        <v>1.333</v>
+        <v>1.357</v>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
@@ -11917,10 +11917,10 @@
         <v>5.4</v>
       </c>
       <c r="J56" t="n">
-        <v>1.877</v>
+        <v>3.05</v>
       </c>
       <c r="K56" t="n">
-        <v>1.877</v>
+        <v>1.357</v>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
@@ -11965,10 +11965,10 @@
         <v>1.6</v>
       </c>
       <c r="J57" t="n">
-        <v>2.55</v>
+        <v>2.9</v>
       </c>
       <c r="K57" t="n">
-        <v>1.476</v>
+        <v>1.385</v>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
@@ -12013,10 +12013,10 @@
         <v>1.4</v>
       </c>
       <c r="J58" t="n">
-        <v>2.8</v>
+        <v>3.05</v>
       </c>
       <c r="K58" t="n">
-        <v>1.408</v>
+        <v>1.357</v>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
@@ -12061,10 +12061,10 @@
         <v>0.6</v>
       </c>
       <c r="J59" t="n">
-        <v>2.55</v>
+        <v>3</v>
       </c>
       <c r="K59" t="n">
-        <v>1.476</v>
+        <v>1.364</v>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
@@ -12157,10 +12157,10 @@
         <v>2.7</v>
       </c>
       <c r="J61" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="K61" t="n">
-        <v>1.435</v>
+        <v>1.364</v>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
@@ -12171,7 +12171,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DeMar DeRozan</t>
+          <t>RJ Barrett</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -12181,45 +12181,45 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>LEAN UNDER</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T3_LEAN</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.542</v>
+        <v>0.527</v>
       </c>
       <c r="F62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>20.7</v>
+        <v>22.6</v>
       </c>
       <c r="I62" t="n">
-        <v>2.2</v>
+        <v>0.1</v>
       </c>
       <c r="J62" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="K62" t="n">
-        <v>1.417</v>
+        <v>1.364</v>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>DeRozan averages 23.0 pts in 3 meetings (+4.5 vs line) — marginally supports the OVER. H2H avg 5.4 pts above season L30; FG% +3.9% trending (L10 vs L30). Opponent is average defense (#13) at slow pace (#25). Mixed signals: 4/10 agree (Context, H2H, FG Trend); counter-signals: Volume, HR L30, HR L10. Projection model targets 20.7 pts (2.2 pts above line; 54% blended confidence [T3]). Risk: high variance (σ=13.8) makes the outcome difficult to call with confidence.</t>
+          <t>[Low conviction — lean only] Barrett's L30 of 19.0 pts sits 3.5 below the 22.5 line — marginally supports the lean UNDER. FG% +5.5% trending (L10 vs L30). Opponent is below-average defense (#16) at moderate pace (#15). Mixed signals: 3/10 agree (Volume, HR L30, Context); counter-signals: HR L10, Trend, Defense. Projection model targets 22.6 pts (0.1 pts above line; 52% blended confidence [T3_LEAN]).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Collin Murray-Boyles</t>
+          <t>DeMar DeRozan</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -12229,7 +12229,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -12238,36 +12238,36 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.632</v>
+        <v>0.542</v>
       </c>
       <c r="F63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>7.5</v>
+        <v>20.7</v>
       </c>
       <c r="I63" t="n">
-        <v>4</v>
+        <v>2.2</v>
       </c>
       <c r="J63" t="n">
-        <v>2.8</v>
+        <v>2.75</v>
       </c>
       <c r="K63" t="n">
-        <v>1.408</v>
+        <v>1.417</v>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>Murray-Boyles's L30 of 8.7 pts sits 2.8 below the 11.5 line — marginally supports the UNDER. FG% +11.6% trending (L10 vs L30); Minutes down 3.5 recently (L10=21.6 vs L30=25.1). Opponent is below-average defense (#16) at moderate pace (#15). Mixed signals: 5/10 agree (Volume, HR L30, HR L10); counter-signals: Trend, Defense, H2H. Projection model targets 7.5 pts (4.0 pts below line; 63% blended confidence [T3]). Risk: minutes trending down (21.6 L10 vs 25.1 L30) — role reduction would suppress counting stats.</t>
+          <t>DeRozan averages 23.0 pts in 3 meetings (+4.5 vs line) — marginally supports the OVER. H2H avg 5.4 pts above season L30; FG% +3.9% trending (L10 vs L30). Opponent is average defense (#13) at slow pace (#25). Mixed signals: 4/10 agree (Context, H2H, FG Trend); counter-signals: Volume, HR L30, HR L10. Projection model targets 20.7 pts (2.2 pts above line; 54% blended confidence [T3]). Risk: high variance (σ=13.8) makes the outcome difficult to call with confidence.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ja'Kobe Walter</t>
+          <t>Collin Murray-Boyles</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -12286,36 +12286,36 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.765</v>
+        <v>0.632</v>
       </c>
       <c r="F64" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G64" t="n">
         <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>-0.5</v>
+        <v>7.5</v>
       </c>
       <c r="I64" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J64" t="n">
-        <v>2.7</v>
+        <v>2.65</v>
       </c>
       <c r="K64" t="n">
-        <v>1.435</v>
+        <v>1.455</v>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Recent scoring trending up 2.9 pts (L5 vs L30) — marginally supports the UNDER. FG% +13.7% trending (L10 vs L30); Minutes up 2.0 recently (L10=23.9 vs L30=21.9). Opponent is weak defense (#25) at moderate pace (#15). Mixed signals: 3/10 agree (Volume, HR L30, Context); counter-signals: HR L10, Trend, Defense. Projection model targets -0.5 pts (11.0 pts below line; 76% blended confidence [T3]).</t>
+          <t>Murray-Boyles's L30 of 8.7 pts sits 2.8 below the 11.5 line — marginally supports the UNDER. FG% +11.6% trending (L10 vs L30); Minutes down 3.5 recently (L10=21.6 vs L30=25.1). Opponent is below-average defense (#16) at moderate pace (#15). Mixed signals: 5/10 agree (Volume, HR L30, HR L10); counter-signals: Trend, Defense, H2H. Projection model targets 7.5 pts (4.0 pts below line; 63% blended confidence [T3]). Risk: minutes trending down (21.6 L10 vs 25.1 L30) — role reduction would suppress counting stats.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RJ Barrett</t>
+          <t>Ja'Kobe Walter</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -12325,7 +12325,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -12334,29 +12334,29 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.539</v>
+        <v>0.765</v>
       </c>
       <c r="F65" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>22.6</v>
+        <v>-0.5</v>
       </c>
       <c r="I65" t="n">
-        <v>1.1</v>
+        <v>11</v>
       </c>
       <c r="J65" t="n">
-        <v>3.15</v>
+        <v>2.6</v>
       </c>
       <c r="K65" t="n">
-        <v>1.333</v>
+        <v>1.465</v>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Barrett's L30 of 19.0 pts sits 2.5 below the 21.5 line — marginally supports the OVER. FG% +5.5% trending (L10 vs L30). Opponent is below-average defense (#16) at moderate pace (#15). Mixed signals: 5/10 agree (HR L10, Trend, Defense); counter-signals: Volume, HR L30, Context. Projection model targets 22.6 pts (1.1 pts above line; 53% blended confidence [T3]). Risk: only 33% hit rate over L30 suggests the line may be set fairly.</t>
+          <t>Recent scoring trending up 2.9 pts (L5 vs L30) — marginally supports the UNDER. FG% +13.7% trending (L10 vs L30); Minutes up 2.0 recently (L10=23.9 vs L30=21.9). Opponent is weak defense (#25) at moderate pace (#15). Mixed signals: 3/10 agree (Volume, HR L30, Context); counter-signals: HR L10, Trend, Defense. Projection model targets -0.5 pts (11.0 pts below line; 76% blended confidence [T3]).</t>
         </is>
       </c>
     </row>
@@ -12397,10 +12397,10 @@
         <v>0.4</v>
       </c>
       <c r="J66" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="K66" t="n">
-        <v>1.385</v>
+        <v>1.408</v>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
@@ -12445,10 +12445,10 @@
         <v>3.1</v>
       </c>
       <c r="J67" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="K67" t="n">
-        <v>1.385</v>
+        <v>1.435</v>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
@@ -12541,10 +12541,10 @@
         <v>3.1</v>
       </c>
       <c r="J69" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="K69" t="n">
-        <v>1.465</v>
+        <v>1.408</v>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
@@ -12589,10 +12589,10 @@
         <v>4.5</v>
       </c>
       <c r="J70" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="K70" t="n">
-        <v>1.435</v>
+        <v>1.385</v>
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
@@ -12637,10 +12637,10 @@
         <v>3.2</v>
       </c>
       <c r="J71" t="n">
-        <v>2.55</v>
+        <v>2.5</v>
       </c>
       <c r="K71" t="n">
-        <v>1.476</v>
+        <v>1.5</v>
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
@@ -12685,10 +12685,10 @@
         <v>4.8</v>
       </c>
       <c r="J72" t="n">
-        <v>2.75</v>
+        <v>2.8</v>
       </c>
       <c r="K72" t="n">
-        <v>1.417</v>
+        <v>1.408</v>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
@@ -12733,10 +12733,10 @@
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>2.85</v>
+        <v>2.7</v>
       </c>
       <c r="K73" t="n">
-        <v>1.4</v>
+        <v>1.435</v>
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
@@ -12766,29 +12766,29 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.554</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="F74" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
       </c>
       <c r="H74" t="n">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I74" t="n">
-        <v>1.6</v>
+        <v>2.7</v>
       </c>
       <c r="J74" t="n">
-        <v>1.769</v>
+        <v>2.7</v>
       </c>
       <c r="K74" t="n">
-        <v>1.98</v>
+        <v>1.435</v>
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>Poeltl's L30 average of 10.5 pts vs the 10.5 line — marginally supports the UNDER. FG% -8.8% trending (L10 vs L30). Opponent is weak defense (#29) at moderate pace (#15). Mixed signals: 4/10 agree (HR L30, Trend, Context); counter-signals: Volume, HR L10, Defense. Projection model targets 8.9 pts (1.6 pts below line; 55% blended confidence [T3]). Risk: high variance (σ=7.1) makes the outcome difficult to call with confidence.</t>
+          <t>Poeltl's L30 average of 10.5 pts vs the 11.5 line — marginally supports the UNDER. FG% -8.8% trending (L10 vs L30). Opponent is weak defense (#29) at moderate pace (#15). Mixed signals: 5/10 agree (Volume, HR L30, Trend); counter-signals: HR L10, Defense, H2H. Projection model targets 8.8 pts (2.7 pts below line; 56% blended confidence [T3]). Risk: high variance (σ=7.1) makes the outcome difficult to call with confidence.</t>
         </is>
       </c>
     </row>
@@ -12829,10 +12829,10 @@
         <v>5.6</v>
       </c>
       <c r="J75" t="n">
-        <v>1.847</v>
+        <v>1.877</v>
       </c>
       <c r="K75" t="n">
-        <v>1.909</v>
+        <v>1.877</v>
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
@@ -12877,10 +12877,10 @@
         <v>0.4</v>
       </c>
       <c r="J76" t="n">
-        <v>1.813</v>
+        <v>1.82</v>
       </c>
       <c r="K76" t="n">
-        <v>1.952</v>
+        <v>1.943</v>
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
@@ -12925,10 +12925,10 @@
         <v>1.3</v>
       </c>
       <c r="J77" t="n">
-        <v>1.8</v>
+        <v>1.926</v>
       </c>
       <c r="K77" t="n">
-        <v>1.971</v>
+        <v>1.833</v>
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
@@ -12973,10 +12973,10 @@
         <v>4.9</v>
       </c>
       <c r="J78" t="n">
-        <v>1.847</v>
+        <v>1.862</v>
       </c>
       <c r="K78" t="n">
-        <v>1.909</v>
+        <v>1.901</v>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
@@ -13021,10 +13021,10 @@
         <v>4.8</v>
       </c>
       <c r="J79" t="n">
-        <v>1.84</v>
+        <v>1.87</v>
       </c>
       <c r="K79" t="n">
-        <v>1.917</v>
+        <v>1.893</v>
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
@@ -13102,7 +13102,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.719</v>
       </c>
       <c r="F81" t="n">
         <v>4</v>
@@ -13114,17 +13114,17 @@
         <v>10.7</v>
       </c>
       <c r="I81" t="n">
-        <v>7.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J81" t="n">
         <v>1.813</v>
       </c>
       <c r="K81" t="n">
-        <v>1.962</v>
+        <v>1.952</v>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>Sexton averages 12.8 pts in 4 meetings (-5.7 vs line) — marginally supports the UNDER. H2H avg 2.3 pts below season L30; TS% shifts -5.1% in this matchup. Opponent is below-average defense (#22) at above-average pace (#12). Mixed signals: 4/10 agree (Volume, HR L30, Context); counter-signals: HR L10, Trend, Defense. Projection model targets 10.7 pts (7.8 pts below line; 68% blended confidence [T3]). Risk: L3 has surged to 22.7 after a 5-pt outing (7.6 above L30) — momentum could push over the under line.</t>
+          <t>Sexton averages 12.8 pts in 4 meetings (-6.7 vs line) — marginally supports the UNDER. H2H avg 2.3 pts below season L30; TS% shifts -5.1% in this matchup. Opponent is below-average defense (#22) at above-average pace (#12). Mixed signals: 4/10 agree (Volume, HR L30, Context); counter-signals: HR L10, Trend, Defense. Projection model targets 10.7 pts (8.8 pts below line; 71% blended confidence [T3]). Risk: L3 has surged to 22.7 after a 5-pt outing (7.6 above L30) — momentum could push over the under line.</t>
         </is>
       </c>
     </row>
@@ -13165,10 +13165,10 @@
         <v>1.7</v>
       </c>
       <c r="J82" t="n">
-        <v>1.87</v>
+        <v>1.877</v>
       </c>
       <c r="K82" t="n">
-        <v>1.893</v>
+        <v>1.877</v>
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
@@ -13213,10 +13213,10 @@
         <v>4.4</v>
       </c>
       <c r="J83" t="n">
-        <v>1.971</v>
+        <v>1.943</v>
       </c>
       <c r="K83" t="n">
-        <v>1.8</v>
+        <v>1.82</v>
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
@@ -13261,10 +13261,10 @@
         <v>1.4</v>
       </c>
       <c r="J84" t="n">
-        <v>1.833</v>
+        <v>1.862</v>
       </c>
       <c r="K84" t="n">
-        <v>1.926</v>
+        <v>1.901</v>
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
@@ -13309,10 +13309,10 @@
         <v>5.3</v>
       </c>
       <c r="J85" t="n">
-        <v>1.971</v>
+        <v>1.926</v>
       </c>
       <c r="K85" t="n">
-        <v>1.8</v>
+        <v>1.833</v>
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
@@ -13357,10 +13357,10 @@
         <v>0.6</v>
       </c>
       <c r="J86" t="n">
-        <v>1.833</v>
+        <v>1.813</v>
       </c>
       <c r="K86" t="n">
-        <v>1.926</v>
+        <v>1.952</v>
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
@@ -13405,10 +13405,10 @@
         <v>3.5</v>
       </c>
       <c r="J87" t="n">
-        <v>1.901</v>
+        <v>1.893</v>
       </c>
       <c r="K87" t="n">
-        <v>1.862</v>
+        <v>1.87</v>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
@@ -13453,10 +13453,10 @@
         <v>2.5</v>
       </c>
       <c r="J88" t="n">
-        <v>1.971</v>
+        <v>1.926</v>
       </c>
       <c r="K88" t="n">
-        <v>1.8</v>
+        <v>1.833</v>
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
@@ -13501,10 +13501,10 @@
         <v>2.6</v>
       </c>
       <c r="J89" t="n">
-        <v>1.877</v>
+        <v>1.893</v>
       </c>
       <c r="K89" t="n">
-        <v>1.877</v>
+        <v>1.87</v>
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
@@ -13549,10 +13549,10 @@
         <v>1.3</v>
       </c>
       <c r="J90" t="n">
-        <v>1.98</v>
+        <v>1.813</v>
       </c>
       <c r="K90" t="n">
-        <v>1.787</v>
+        <v>1.952</v>
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
@@ -13597,10 +13597,10 @@
         <v>2.5</v>
       </c>
       <c r="J91" t="n">
-        <v>1.943</v>
+        <v>1.917</v>
       </c>
       <c r="K91" t="n">
-        <v>1.82</v>
+        <v>1.84</v>
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
@@ -13645,10 +13645,10 @@
         <v>3</v>
       </c>
       <c r="J92" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="K92" t="n">
         <v>1.893</v>
-      </c>
-      <c r="K92" t="n">
-        <v>1.87</v>
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
@@ -13741,10 +13741,10 @@
         <v>0.6</v>
       </c>
       <c r="J94" t="n">
-        <v>1.84</v>
+        <v>1.943</v>
       </c>
       <c r="K94" t="n">
-        <v>1.917</v>
+        <v>1.82</v>
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
@@ -13789,10 +13789,10 @@
         <v>1.2</v>
       </c>
       <c r="J95" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="K95" t="n">
-        <v>1.781</v>
+        <v>1.769</v>
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
@@ -13837,10 +13837,10 @@
         <v>4.7</v>
       </c>
       <c r="J96" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="K96" t="n">
-        <v>1.787</v>
+        <v>1.769</v>
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
@@ -13885,10 +13885,10 @@
         <v>1.5</v>
       </c>
       <c r="J97" t="n">
-        <v>1.84</v>
+        <v>1.82</v>
       </c>
       <c r="K97" t="n">
-        <v>1.917</v>
+        <v>1.943</v>
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
@@ -13981,10 +13981,10 @@
         <v>2</v>
       </c>
       <c r="J99" t="n">
-        <v>1.84</v>
+        <v>1.833</v>
       </c>
       <c r="K99" t="n">
-        <v>1.917</v>
+        <v>1.926</v>
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
@@ -14029,10 +14029,10 @@
         <v>1.9</v>
       </c>
       <c r="J100" t="n">
-        <v>1.926</v>
+        <v>1.99</v>
       </c>
       <c r="K100" t="n">
-        <v>1.833</v>
+        <v>1.781</v>
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
@@ -14077,10 +14077,10 @@
         <v>1.9</v>
       </c>
       <c r="J101" t="n">
-        <v>1.877</v>
+        <v>1.847</v>
       </c>
       <c r="K101" t="n">
-        <v>1.877</v>
+        <v>1.909</v>
       </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
@@ -14125,10 +14125,10 @@
         <v>3.1</v>
       </c>
       <c r="J102" t="n">
-        <v>1.893</v>
+        <v>1.877</v>
       </c>
       <c r="K102" t="n">
-        <v>1.87</v>
+        <v>1.877</v>
       </c>
       <c r="L102" s="2" t="inlineStr">
         <is>
@@ -14173,10 +14173,10 @@
         <v>4.8</v>
       </c>
       <c r="J103" t="n">
-        <v>1.901</v>
+        <v>1.893</v>
       </c>
       <c r="K103" t="n">
-        <v>1.862</v>
+        <v>1.87</v>
       </c>
       <c r="L103" s="2" t="inlineStr">
         <is>
@@ -14269,10 +14269,10 @@
         <v>0.3</v>
       </c>
       <c r="J105" t="n">
+        <v>1.862</v>
+      </c>
+      <c r="K105" t="n">
         <v>1.901</v>
-      </c>
-      <c r="K105" t="n">
-        <v>1.862</v>
       </c>
       <c r="L105" s="2" t="inlineStr">
         <is>
@@ -14413,10 +14413,10 @@
         <v>3.3</v>
       </c>
       <c r="J108" t="n">
-        <v>1.943</v>
+        <v>1.917</v>
       </c>
       <c r="K108" t="n">
-        <v>1.82</v>
+        <v>1.84</v>
       </c>
       <c r="L108" s="2" t="inlineStr">
         <is>
@@ -14567,7 +14567,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>19.5</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="6">
@@ -14647,7 +14647,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="10">
@@ -14733,7 +14733,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jevon Carter</t>
+          <t>Franz Wagner</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -14747,7 +14747,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>8.5</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="15">
@@ -14967,7 +14967,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="26">
@@ -15333,7 +15333,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kevin Durant</t>
+          <t>Jabari Smith Jr.</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -15343,17 +15343,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>25.5</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jabari Smith Jr.</t>
+          <t>Kevin Durant</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -15363,11 +15363,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>16.5</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="46">
@@ -15393,7 +15393,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tari Eason</t>
+          <t>Gary Trent Jr.</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -15407,13 +15407,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>9.5</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Gary Trent Jr.</t>
+          <t>Tari Eason</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -15427,7 +15427,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>13.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="49">
@@ -15693,7 +15693,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DeMar DeRozan</t>
+          <t>RJ Barrett</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -15703,17 +15703,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>LEAN UNDER</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>18.5</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Collin Murray-Boyles</t>
+          <t>DeMar DeRozan</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -15723,17 +15723,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>11.5</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ja'Kobe Walter</t>
+          <t>Collin Murray-Boyles</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -15747,13 +15747,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RJ Barrett</t>
+          <t>Ja'Kobe Walter</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -15763,11 +15763,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>21.5</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="66">
@@ -15947,7 +15947,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="75">
@@ -16087,7 +16087,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="82">

</xml_diff>